<commit_message>
dodanie nazw kolumn w wynikowej csv
</commit_message>
<xml_diff>
--- a/dane.xlsx
+++ b/dane.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dorot\OneDrive\Desktop\Praca naukowa\Ochrona środowiska\ochrona_srod\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kosa1\PycharmProjects\ekosystem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B2E5E47-5471-4026-B82D-0BA4F8C01F03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{496E7E08-7891-4C96-9823-88E93870FD96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5940" yWindow="3396" windowWidth="14580" windowHeight="7548" xr2:uid="{3CA7BE9C-EA14-4A95-AF0E-A6C58FEAE276}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="5" xr2:uid="{3CA7BE9C-EA14-4A95-AF0E-A6C58FEAE276}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="6" r:id="rId1"/>
@@ -23,7 +23,20 @@
   <definedNames>
     <definedName name="_xlnm.Database">'5.1. Woda'!$A$1:$AE$215</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -44901,7 +44914,7 @@
       <c r="C10" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="2">
         <v>1</v>
       </c>
       <c r="E10" s="2" t="s">

</xml_diff>

<commit_message>
zmiana nazwy atrybutu woda na jednolitą z pozostałymi grupami
</commit_message>
<xml_diff>
--- a/dane.xlsx
+++ b/dane.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kosa1\PycharmProjects\ekosystem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{496E7E08-7891-4C96-9823-88E93870FD96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38984A72-D825-4344-9BDB-AA687816E6F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="5" xr2:uid="{3CA7BE9C-EA14-4A95-AF0E-A6C58FEAE276}"/>
+    <workbookView xWindow="4812" yWindow="1548" windowWidth="17280" windowHeight="9960" activeTab="1" xr2:uid="{3CA7BE9C-EA14-4A95-AF0E-A6C58FEAE276}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="6" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8082" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8082" uniqueCount="262">
   <si>
     <t>R3W1_LS</t>
   </si>
@@ -897,9 +897,6 @@
   </si>
   <si>
     <t>Name</t>
-  </si>
-  <si>
-    <t>R1W4 LS</t>
   </si>
 </sst>
 </file>
@@ -1921,7 +1918,7 @@
         <v>22</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>262</v>
+        <v>23</v>
       </c>
       <c r="Z1" s="1" t="s">
         <v>24</v>

</xml_diff>